<commit_message>
feat(budget): voci di spesa, lettura di tutti i documenti, budget dall'azienda e dall'allocazione
- tassonomia di oltre 50 voci di spesa sotto le cinque categorie; i bandi possono escludere una voce per nome (regola estratta dal testo con la frase come prova, controllo 16, stima, allocazione)
- lettura dei fogli Excel (organico, cespiti, fatture, budget, investimenti, assunzioni, aiuti) e dei PDF con dati precisi (DURC, locazione, credito R&S, finanziamento); nome e codice fiscale non entrano mai
- bozza di budget: personale persona per persona, spese per voce con fonte (budget aziendale, piano investimenti, previsione), niente ammortamento
- allocazione per voce con aiuto cumulato massimo; budget di ogni bando ricavato dall'allocazione, verificato da solo e insieme agli altri, apribile nella pagina Budget
- azienda di prova: 50 documenti (17 cedolini coerenti con il registro del personale)
- test 523, documenti aggiornati

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documenti_di_prova/meridiana_digital_solutions/14_Organico_e_livelli_CCNL.xlsx
+++ b/documenti_di_prova/meridiana_digital_solutions/14_Organico_e_livelli_CCNL.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Piano assunzioni 2026-28" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Organico'!$A$1:$R$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Organico'!$A$1:$S$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Retribuzioni lorde 2025'!$A$1:$O$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Costo del lavoro 2025'!$A$1:$G$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cedolini 2026 (lordo)'!$A$1:$L$18</definedName>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -491,6 +491,7 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="48" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -584,6 +585,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>CCNL applicato</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -659,6 +665,11 @@
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -734,6 +745,11 @@
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -809,6 +825,11 @@
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -884,6 +905,11 @@
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -959,6 +985,11 @@
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1034,6 +1065,11 @@
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1109,6 +1145,11 @@
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1184,6 +1225,11 @@
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1259,6 +1305,11 @@
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1334,6 +1385,11 @@
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1413,6 +1469,11 @@
           <t>Part time 75%</t>
         </is>
       </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1488,6 +1549,11 @@
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1567,6 +1633,11 @@
           <t>Apprendistato professionalizzante</t>
         </is>
       </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1642,6 +1713,11 @@
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1717,6 +1793,11 @@
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1796,6 +1877,11 @@
           <t>Apprendistato professionalizzante</t>
         </is>
       </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1873,6 +1959,11 @@
       <c r="R18" s="2" t="inlineStr">
         <is>
           <t>Apprendistato professionalizzante</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>CCNL Commercio, Terziario Distribuzione e Servizi (Confcommercio)</t>
         </is>
       </c>
     </row>
@@ -1905,9 +1996,10 @@
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="n"/>
       <c r="R19" s="7" t="n"/>
+      <c r="S19" s="7" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R18"/>
+  <autoFilter ref="A1:S18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3627,35 +3719,35 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>8171.42</v>
+        <v>8071.42</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>4085.71</v>
+        <v>4035.71</v>
       </c>
       <c r="K2" s="5">
         <f>SUM(C2:J2)</f>
         <v/>
       </c>
       <c r="L2" s="2" t="n">
-        <v>2544.03</v>
+        <v>2519.32</v>
       </c>
     </row>
     <row r="3">
@@ -3670,35 +3762,35 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>7228.58</v>
+        <v>7142.86</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>3614.29</v>
+        <v>3571.43</v>
       </c>
       <c r="K3" s="5">
         <f>SUM(C3:J3)</f>
         <v/>
       </c>
       <c r="L3" s="2" t="n">
-        <v>2313.12</v>
+        <v>2292.2</v>
       </c>
     </row>
     <row r="4">
@@ -3713,35 +3805,35 @@
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>5961.54</v>
+        <v>5900</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>2980.77</v>
+        <v>2950</v>
       </c>
       <c r="K4" s="5">
         <f>SUM(C4:J4)</f>
         <v/>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2004.09</v>
+        <v>1989.08</v>
       </c>
     </row>
     <row r="5">
@@ -3756,35 +3848,35 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>5919.04</v>
+        <v>5842.86</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>2959.52</v>
+        <v>2921.43</v>
       </c>
       <c r="K5" s="5">
         <f>SUM(C5:J5)</f>
         <v/>
       </c>
       <c r="L5" s="2" t="n">
-        <v>1993.72</v>
+        <v>1975.13</v>
       </c>
     </row>
     <row r="6">
@@ -3799,35 +3891,35 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>5185.72</v>
+        <v>5128.58</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>2592.86</v>
+        <v>2564.29</v>
       </c>
       <c r="K6" s="5">
         <f>SUM(C6:J6)</f>
         <v/>
       </c>
       <c r="L6" s="2" t="n">
-        <v>1814.86</v>
+        <v>1800.93</v>
       </c>
     </row>
     <row r="7">
@@ -3842,35 +3934,35 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>5128.2</v>
+        <v>5057.14</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>2564.1</v>
+        <v>2528.57</v>
       </c>
       <c r="K7" s="5">
         <f>SUM(C7:J7)</f>
         <v/>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1800.83</v>
+        <v>1783.5</v>
       </c>
     </row>
     <row r="8">
@@ -3885,35 +3977,35 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>5028.58</v>
+        <v>4971.42</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>2514.29</v>
+        <v>2485.71</v>
       </c>
       <c r="K8" s="5">
         <f>SUM(C8:J8)</f>
         <v/>
       </c>
       <c r="L8" s="2" t="n">
-        <v>1776.54</v>
+        <v>1762.59</v>
       </c>
     </row>
     <row r="9">
@@ -3928,35 +4020,35 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>6390.48</v>
+        <v>6314.28</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>3195.24</v>
+        <v>3157.14</v>
       </c>
       <c r="K9" s="5">
         <f>SUM(C9:J9)</f>
         <v/>
       </c>
       <c r="L9" s="2" t="n">
-        <v>2108.7</v>
+        <v>2090.12</v>
       </c>
     </row>
     <row r="10">
@@ -3971,35 +4063,35 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>4976.2</v>
+        <v>4914.28</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>2488.1</v>
+        <v>2457.14</v>
       </c>
       <c r="K10" s="5">
         <f>SUM(C10:J10)</f>
         <v/>
       </c>
       <c r="L10" s="2" t="n">
-        <v>1763.76</v>
+        <v>1748.64</v>
       </c>
     </row>
     <row r="11">
@@ -4014,35 +4106,35 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>4923.8</v>
+        <v>4871.42</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>2461.9</v>
+        <v>2435.71</v>
       </c>
       <c r="K11" s="5">
         <f>SUM(C11:J11)</f>
         <v/>
       </c>
       <c r="L11" s="2" t="n">
-        <v>1750.98</v>
+        <v>1738.21</v>
       </c>
     </row>
     <row r="12">
@@ -4057,35 +4149,35 @@
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>3509.52</v>
+        <v>3471.42</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>1754.76</v>
+        <v>1735.71</v>
       </c>
       <c r="K12" s="5">
         <f>SUM(C12:J12)</f>
         <v/>
       </c>
       <c r="L12" s="2" t="n">
-        <v>1359.17</v>
+        <v>1347.89</v>
       </c>
     </row>
     <row r="13">
@@ -4100,35 +4192,35 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>4871.42</v>
+        <v>4814.28</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>2435.71</v>
+        <v>2407.14</v>
       </c>
       <c r="K13" s="5">
         <f>SUM(C13:J13)</f>
         <v/>
       </c>
       <c r="L13" s="2" t="n">
-        <v>1738.21</v>
+        <v>1724.27</v>
       </c>
     </row>
     <row r="14">
@@ -4143,35 +4235,35 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>3855.24</v>
+        <v>3814.28</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>1927.62</v>
+        <v>1907.14</v>
       </c>
       <c r="K14" s="5">
         <f>SUM(C14:J14)</f>
         <v/>
       </c>
       <c r="L14" s="2" t="n">
-        <v>1461.59</v>
+        <v>1449.46</v>
       </c>
     </row>
     <row r="15">
@@ -4186,35 +4278,35 @@
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>5814.28</v>
+        <v>5742.86</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>2907.14</v>
+        <v>2871.43</v>
       </c>
       <c r="K15" s="5">
         <f>SUM(C15:J15)</f>
         <v/>
       </c>
       <c r="L15" s="2" t="n">
-        <v>1968.17</v>
+        <v>1950.75</v>
       </c>
     </row>
     <row r="16">
@@ -4229,35 +4321,35 @@
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>5657.14</v>
+        <v>5585.72</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>2828.57</v>
+        <v>2792.86</v>
       </c>
       <c r="K16" s="5">
         <f>SUM(C16:J16)</f>
         <v/>
       </c>
       <c r="L16" s="2" t="n">
-        <v>1929.84</v>
+        <v>1912.43</v>
       </c>
     </row>
     <row r="17">
@@ -4272,35 +4364,35 @@
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>3771.42</v>
+        <v>3728.58</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>1885.71</v>
+        <v>1864.29</v>
       </c>
       <c r="K17" s="5">
         <f>SUM(C17:J17)</f>
         <v/>
       </c>
       <c r="L17" s="2" t="n">
-        <v>1436.76</v>
+        <v>1424.06</v>
       </c>
     </row>
     <row r="18">
@@ -4318,32 +4410,32 @@
         <v>0</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>1859.52</v>
+        <v>1835.71</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>1859.52</v>
+        <v>1835.71</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>1859.52</v>
+        <v>1835.71</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1859.52</v>
+        <v>1835.71</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>3719.04</v>
+        <v>3671.42</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1859.52</v>
+        <v>1835.71</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>1859.52</v>
+        <v>1835.71</v>
       </c>
       <c r="K18" s="5">
         <f>SUM(C18:J18)</f>
         <v/>
       </c>
       <c r="L18" s="2" t="n">
-        <v>1421.25</v>
+        <v>1407.14</v>
       </c>
     </row>
     <row r="19">

</xml_diff>